<commit_message>
Load Census data and join to dfCapLastGrade.
</commit_message>
<xml_diff>
--- a/project_tracking.xlsx
+++ b/project_tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/942f786d6b81c97a/_JHU/Capstone/capstone/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="217" documentId="8_{3422572A-D085-42D3-912D-81DD938225BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{363763CA-CE37-44D3-A08B-3E0BB1231E0B}"/>
+  <xr:revisionPtr revIDLastSave="281" documentId="8_{3422572A-D085-42D3-912D-81DD938225BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E35DE08-2B00-499E-9AE0-3090A710F8AF}"/>
   <bookViews>
-    <workbookView xWindow="56595" yWindow="1155" windowWidth="30210" windowHeight="18615" activeTab="2" xr2:uid="{91F703DA-BFA0-4E62-9200-A6AD10BEA7A1}"/>
+    <workbookView minimized="1" xWindow="41925" yWindow="3990" windowWidth="20160" windowHeight="15390" activeTab="1" xr2:uid="{91F703DA-BFA0-4E62-9200-A6AD10BEA7A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Files" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="173">
   <si>
     <t>american-political-science-association.csl</t>
   </si>
@@ -130,15 +130,9 @@
     <t>Morse_Capstone_Proposal.qmd</t>
   </si>
   <si>
-    <t>Quarto file used to generate Porject Proposal turned in on 2/6/2026.</t>
-  </si>
-  <si>
     <t>Morse_Capstone.qmd</t>
   </si>
   <si>
-    <t>Duplication of paper_template.qmd</t>
-  </si>
-  <si>
     <t>panel.R</t>
   </si>
   <si>
@@ -182,9 +176,6 @@
   </si>
   <si>
     <t>validate-data.R</t>
-  </si>
-  <si>
-    <t>Used to validate the source data was loaded correctly.</t>
   </si>
   <si>
     <t>project_tracking.xlsx</t>
@@ -419,9 +410,6 @@
     <t>district_directory.rds</t>
   </si>
   <si>
-    <t>Necessary code copied into load-data.R. Loads and consolidates raw CSV files for source data for enrollment outcomes and WA school directory. Creates data frames and stores as RDS files.</t>
-  </si>
-  <si>
     <t>Column</t>
   </si>
   <si>
@@ -570,6 +558,81 @@
   </si>
   <si>
     <t>entity-fixed effect</t>
+  </si>
+  <si>
+    <t>ela_score</t>
+  </si>
+  <si>
+    <t>ela_female_score</t>
+  </si>
+  <si>
+    <t>ela_li_score</t>
+  </si>
+  <si>
+    <t>math_score</t>
+  </si>
+  <si>
+    <t>math_li_score</t>
+  </si>
+  <si>
+    <t>math_female_score</t>
+  </si>
+  <si>
+    <t>Weighted score based on logit transformation of SBAC ELA performance. Most weight applied to 11th grade results, least weight applied to 3rd grade.</t>
+  </si>
+  <si>
+    <t>Weighted score based on logit transformation of SBAC ELA performance for Low Income students. Most weight applied to 11th grade results, least weight applied to 3rd grade.</t>
+  </si>
+  <si>
+    <t>Weighted score based on logit transformation of SBAC ELA performance for Female students. Most weight applied to 11th grade results, least weight applied to 3rd grade.</t>
+  </si>
+  <si>
+    <t>Weighted score based on logit transformation of SBAC Math performance. Most weight applied to 11th grade results, least weight applied to 3rd grade.</t>
+  </si>
+  <si>
+    <t>Weighted score based on logit transformation of SBAC Math performance for Low Income students. Most weight applied to 11th grade results, least weight applied to 3rd grade.</t>
+  </si>
+  <si>
+    <t>Weighted score based on logit transformation of SBAC Math performance for Female students. Most weight applied to 11th grade results, least weight applied to 3rd grade.</t>
+  </si>
+  <si>
+    <t>Used to design various charts and analyses for the final document. All analyses are recreated in the Quarto file.</t>
+  </si>
+  <si>
+    <t>analysis2.R</t>
+  </si>
+  <si>
+    <t>Used to design the regression analyses for the final document. All analyses are recreated in the Quarto file.</t>
+  </si>
+  <si>
+    <t>Used to design the datasets used for build-dataset.R.</t>
+  </si>
+  <si>
+    <t>build-county-dataset.R</t>
+  </si>
+  <si>
+    <t>Aggregates the data to County level, specifically for use in Mapping visualizations.</t>
+  </si>
+  <si>
+    <t>Removed</t>
+  </si>
+  <si>
+    <t>Quarto file used to generate Project Proposal turned in on 2/6/2026.</t>
+  </si>
+  <si>
+    <t>Removed. Duplication of paper_template.qmd</t>
+  </si>
+  <si>
+    <t>Removed. Used to validate the source data was loaded correctly.</t>
+  </si>
+  <si>
+    <t>Removed. Necessary code copied into load-data.R. Loads and consolidates raw CSV files for source data for enrollment outcomes and WA school directory. Creates data frames and stores as RDS files.</t>
+  </si>
+  <si>
+    <t>load-census-data.R</t>
+  </si>
+  <si>
+    <t>Loads and consolidates raw CSV files downloaded from the US Census Bureau.</t>
   </si>
 </sst>
 </file>
@@ -658,22 +721,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -694,7 +742,22 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -710,28 +773,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8D427B93-56E7-4F2F-9853-C8EBF42EAE8B}" name="Table1" displayName="Table1" ref="A1:D24" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
-  <autoFilter ref="A1:D24" xr:uid="{8D427B93-56E7-4F2F-9853-C8EBF42EAE8B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8D427B93-56E7-4F2F-9853-C8EBF42EAE8B}" name="Table1" displayName="Table1" ref="A1:D27" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="A1:D27" xr:uid="{8D427B93-56E7-4F2F-9853-C8EBF42EAE8B}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{668D53DB-5951-4D87-8902-1BD236B2A8CC}" name="File" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{27A06D4B-4A80-43E3-8089-FF5099989DB4}" name="File Type" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{3D72D5BF-A3F1-438B-A127-FEA4D5287CC8}" name="Required" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{0C7FA01E-3A90-4CC4-9F30-46CA136BE87E}" name="Description" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{668D53DB-5951-4D87-8902-1BD236B2A8CC}" name="File" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{27A06D4B-4A80-43E3-8089-FF5099989DB4}" name="File Type" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{3D72D5BF-A3F1-438B-A127-FEA4D5287CC8}" name="Required" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{0C7FA01E-3A90-4CC4-9F30-46CA136BE87E}" name="Description" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3CAFBC2B-DEE9-4317-9903-B30AF5BA6CE5}" name="Table2" displayName="Table2" ref="A1:F13" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3CAFBC2B-DEE9-4317-9903-B30AF5BA6CE5}" name="Table2" displayName="Table2" ref="A1:F13" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
   <autoFilter ref="A1:F13" xr:uid="{3CAFBC2B-DEE9-4317-9903-B30AF5BA6CE5}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{42C72726-126A-4572-9516-35A0889CB916}" name="Subject" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{48F1C3D7-E092-47A1-ACF2-0CF5AD85CB38}" name="RDS File" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{87D0CCDD-0F3D-406A-BB87-6348C0288853}" name="File Name (as downloaded)" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{76513B85-9BB0-4878-A632-2C577C6B2AD8}" name="File Name (renamed for project)" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{55C06612-5DCB-4D87-B42E-6971DAC54A05}" name="URL" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{25154F36-5FC0-47EE-B275-8E34F1D4E1C1}" name="Description" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{42C72726-126A-4572-9516-35A0889CB916}" name="Subject" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{48F1C3D7-E092-47A1-ACF2-0CF5AD85CB38}" name="RDS File" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{87D0CCDD-0F3D-406A-BB87-6348C0288853}" name="File Name (as downloaded)" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{76513B85-9BB0-4878-A632-2C577C6B2AD8}" name="File Name (renamed for project)" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{55C06612-5DCB-4D87-B42E-6971DAC54A05}" name="URL" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{25154F36-5FC0-47EE-B275-8E34F1D4E1C1}" name="Description" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1054,7 +1117,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48A345CD-4AD3-411B-8FA1-AF0BD1EB1B2E}">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="38.26953125" style="1" bestFit="1" customWidth="1"/>
@@ -1092,103 +1155,115 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" ht="29">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="C3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="29">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>161</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="C4" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="D4" s="2" t="s">
-        <v>7</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="D5" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>10</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="29">
       <c r="A8" s="1" t="s">
-        <v>13</v>
+        <v>164</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>15</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="29">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="58">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>5</v>
@@ -1197,68 +1272,68 @@
         <v>17</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="29">
       <c r="A12" s="1" t="s">
-        <v>21</v>
+        <v>171</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>28</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="29">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="58">
       <c r="A14" s="1" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>32</v>
+        <v>170</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="29">
       <c r="A16" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>22</v>
@@ -1267,110 +1342,110 @@
         <v>17</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>36</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="1" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="29">
+      <c r="A19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="29">
-      <c r="A18" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="29">
-      <c r="A20" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="D20" s="2" t="s">
-        <v>92</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="29">
       <c r="A21" s="1" t="s">
-        <v>99</v>
+        <v>35</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>93</v>
+        <v>37</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="29">
       <c r="A23" s="1" t="s">
-        <v>45</v>
+        <v>88</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="29">
       <c r="A24" s="1" t="s">
-        <v>47</v>
+        <v>96</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>5</v>
@@ -1379,7 +1454,49 @@
         <v>17</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>48</v>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="29">
+      <c r="A26" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="29">
+      <c r="A27" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -1405,19 +1522,19 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>27</v>
@@ -1425,212 +1542,212 @@
     </row>
     <row r="2" spans="1:6" ht="58">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="58">
       <c r="A3" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="72.5">
       <c r="A4" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="72.5">
       <c r="A5" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>64</v>
-      </c>
       <c r="F5" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="72.5">
       <c r="A6" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="72.5">
       <c r="A7" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="72.5">
       <c r="A8" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="72.5">
       <c r="A9" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="72.5">
       <c r="A10" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="72.5">
       <c r="A11" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="58">
       <c r="A12" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>82</v>
-      </c>
       <c r="E12" s="3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="43.5">
       <c r="A13" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1655,7 +1772,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1AB036A-0EB6-4FE4-A99C-870523E2733D}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="16.90625" bestFit="1" customWidth="1"/>
@@ -1665,13 +1782,13 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>27</v>
@@ -1679,282 +1796,366 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C2" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="D3" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B4" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C4" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B5" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C5" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C6" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="D6" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>115</v>
+        <v>135</v>
       </c>
       <c r="B7" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C7" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D7" t="s">
-        <v>116</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
       <c r="B8" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C8" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D8" t="s">
-        <v>118</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>119</v>
+        <v>137</v>
       </c>
       <c r="B9" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D9" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="B10" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C10" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D10" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="B11" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C11" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D11" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B12" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C12" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="B13" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C13" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D13" t="s">
-        <v>126</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="B14" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C14" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D14" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="B15" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C15" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D15" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="B16" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C16" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D16" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="B17" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C17" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D17" t="s">
-        <v>136</v>
+        <v>156</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="B18" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C18" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D18" t="s">
-        <v>138</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="B19" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C19" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D19" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>140</v>
+        <v>119</v>
       </c>
       <c r="B20" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C20" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D20" t="s">
-        <v>143</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="B21" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C21" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D21" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B22" t="s">
+        <v>104</v>
+      </c>
+      <c r="C22" t="s">
         <v>144</v>
+      </c>
+      <c r="D22" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" t="s">
+        <v>153</v>
+      </c>
+      <c r="B23" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" t="s">
+        <v>144</v>
+      </c>
+      <c r="D23" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" t="s">
+        <v>104</v>
+      </c>
+      <c r="C24" t="s">
+        <v>144</v>
+      </c>
+      <c r="D24" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" t="s">
+        <v>129</v>
+      </c>
+      <c r="B25" t="s">
+        <v>104</v>
+      </c>
+      <c r="C25" t="s">
+        <v>144</v>
+      </c>
+      <c r="D25" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" t="s">
+        <v>144</v>
+      </c>
+      <c r="D26" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" t="s">
+        <v>133</v>
+      </c>
+      <c r="B27" t="s">
+        <v>104</v>
+      </c>
+      <c r="C27" t="s">
+        <v>144</v>
+      </c>
+      <c r="D27" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>